<commit_message>
style(frontend): revamp GeoFencingMenu and GeoFencingTag to fix layout issues and add Medorn-style UI
</commit_message>
<xml_diff>
--- a/REPORTING MODULE/city-area.xlsx
+++ b/REPORTING MODULE/city-area.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MY WORK FLOW\Emyris Onboard App\REPORTING MODULE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2449712B-A383-4D4C-B6E9-4D11FB072EFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04A90981-DF41-4DA9-9C67-3A9ACBD1D9DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1272,12 +1272,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F144"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="21.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1297,7 +1298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1314,7 +1315,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1348,7 +1349,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1365,7 +1366,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1382,7 +1383,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1399,7 +1400,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1433,7 +1434,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1450,7 +1451,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1467,7 +1468,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1484,7 +1485,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1501,7 +1502,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1518,7 +1519,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1535,7 +1536,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1552,7 +1553,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1586,7 +1587,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1603,7 +1604,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1620,7 +1621,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1654,7 +1655,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1671,7 +1672,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1688,7 +1689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1705,7 +1706,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1722,7 +1723,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1739,7 +1740,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1756,7 +1757,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1773,7 +1774,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1790,7 +1791,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1824,7 +1825,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1841,7 +1842,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1858,7 +1859,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1875,7 +1876,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1892,7 +1893,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1909,7 +1910,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1926,7 +1927,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1943,7 +1944,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1960,7 +1961,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1977,7 +1978,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1994,7 +1995,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2011,7 +2012,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2028,7 +2029,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2045,7 +2046,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2062,7 +2063,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2079,7 +2080,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2096,7 +2097,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2130,7 +2131,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2147,7 +2148,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2164,7 +2165,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2181,7 +2182,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2198,7 +2199,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2215,7 +2216,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2232,7 +2233,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2249,7 +2250,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2266,7 +2267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2283,7 +2284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2300,7 +2301,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2317,7 +2318,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2334,7 +2335,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2351,7 +2352,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2368,7 +2369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2385,7 +2386,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2402,7 +2403,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2419,7 +2420,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2436,7 +2437,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2453,7 +2454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2470,7 +2471,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2487,7 +2488,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2504,7 +2505,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2521,7 +2522,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2538,7 +2539,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2555,7 +2556,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2572,7 +2573,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2589,7 +2590,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2606,7 +2607,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2623,7 +2624,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2640,7 +2641,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2657,7 +2658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2674,7 +2675,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2691,7 +2692,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2708,7 +2709,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2725,7 +2726,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2742,7 +2743,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2759,7 +2760,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2776,7 +2777,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2793,7 +2794,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2810,7 +2811,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2827,7 +2828,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2844,7 +2845,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2861,7 +2862,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2878,7 +2879,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2895,7 +2896,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2912,7 +2913,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2929,7 +2930,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2963,7 +2964,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2980,7 +2981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3014,7 +3015,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3031,7 +3032,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3048,7 +3049,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3065,7 +3066,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3082,7 +3083,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3099,7 +3100,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3116,7 +3117,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3133,7 +3134,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3150,7 +3151,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3167,7 +3168,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3184,7 +3185,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -3201,7 +3202,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -3218,7 +3219,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -3235,7 +3236,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -3252,7 +3253,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -3269,7 +3270,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -3286,7 +3287,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -3303,7 +3304,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -3320,7 +3321,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -3337,7 +3338,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -3354,7 +3355,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -3371,7 +3372,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -3388,7 +3389,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -3405,7 +3406,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -3422,7 +3423,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -3439,7 +3440,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3456,7 +3457,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3473,7 +3474,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3490,7 +3491,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="131" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>130</v>
       </c>
@@ -3507,23 +3508,22 @@
         <v>127</v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="15.75" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="143" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="144" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>289</v>
       </c>

</xml_diff>